<commit_message>
Format LME032 validation hyperlinks blue and underlined
</commit_message>
<xml_diff>
--- a/regions/LME_032/LME032_taxon_mapping_appendix.xlsx
+++ b/regions/LME_032/LME032_taxon_mapping_appendix.xlsx
@@ -23,7 +23,7 @@
     <x:numFmt numFmtId="203" formatCode="#,##0.000000"/>
     <x:numFmt numFmtId="204" formatCode="0.0000%"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -50,6 +50,12 @@
       <x:color rgb="FF0563C1"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Calibri"/>
+      <x:color rgb="FF0563C1"/>
+      <x:u val="single"/>
+    </x:font>
   </x:fonts>
   <x:fills count="3">
     <x:fill>
@@ -70,7 +76,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -122,6 +128,9 @@
       <x:alignment vertical="top"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -13691,7 +13700,7 @@
       <x:c r="C5" s="9" t="str">
         <x:v>Membership pp. 11–20/PDF 21–30; landings p. 13/PDF 23; zero BA and basic inputs p. 21/PDF 31; balanced diet p. 53/PDF 63; area p. 8/PDF 18.</x:v>
       </x:c>
-      <x:c r="D5" s="18" t="str">
+      <x:c r="D5" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13705,7 +13714,7 @@
       <x:c r="C6" s="9" t="str">
         <x:v>CMFRI repository; inspected 30 September 2026</x:v>
       </x:c>
-      <x:c r="D6" s="18" t="str">
+      <x:c r="D6" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13719,7 +13728,7 @@
       <x:c r="C7" s="9" t="str">
         <x:v>Catch; Classic PPR/Taxa; independent annual method treatment.</x:v>
       </x:c>
-      <x:c r="D7" s="18" t="str">
+      <x:c r="D7" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13733,7 +13742,7 @@
       <x:c r="C8" s="9" t="str">
         <x:v>Sea Around Us API frozen source, catalogued 3 September 2026.</x:v>
       </x:c>
-      <x:c r="D8" s="18" t="str">
+      <x:c r="D8" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13747,7 +13756,7 @@
       <x:c r="C9" s="9" t="str">
         <x:v>Sea Around Us regional exploited-organisms snapshot.</x:v>
       </x:c>
-      <x:c r="D9" s="18" t="str">
+      <x:c r="D9" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13761,7 +13770,7 @@
       <x:c r="C10" s="9" t="str">
         <x:v>Common taxonomic reference provenance.</x:v>
       </x:c>
-      <x:c r="D10" s="18" t="str">
+      <x:c r="D10" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13775,7 +13784,7 @@
       <x:c r="C11" s="9" t="str">
         <x:v>475 exact records from 517 queried taxon/source names; retrieved 30 September 2026.</x:v>
       </x:c>
-      <x:c r="D11" s="18" t="str">
+      <x:c r="D11" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13789,7 +13798,7 @@
       <x:c r="C12" s="9" t="str">
         <x:v>Keyed adopted audit; concise appendix derives from these same rows.</x:v>
       </x:c>
-      <x:c r="D12" s="18" t="str">
+      <x:c r="D12" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13803,7 +13812,7 @@
       <x:c r="C13" s="9" t="str">
         <x:v>Source/model allocation and retained-weight reconstruction.</x:v>
       </x:c>
-      <x:c r="D13" s="18" t="str">
+      <x:c r="D13" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13817,7 +13826,7 @@
       <x:c r="C14" s="9" t="str">
         <x:v>Sailfish 0–200 m and fish/squid predation; swordfish wider depth use. Retrieved 30 September 2026.</x:v>
       </x:c>
-      <x:c r="D14" s="18" t="str">
+      <x:c r="D14" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13831,7 +13840,7 @@
       <x:c r="C15" s="9" t="str">
         <x:v>FishBase Xiphias gladius; retrieved 30 September 2026.</x:v>
       </x:c>
-      <x:c r="D15" s="18" t="str">
+      <x:c r="D15" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13845,7 +13854,7 @@
       <x:c r="C16" s="9" t="str">
         <x:v>FishBase/FAO Collette(1999), retrieved 30 September 2026.</x:v>
       </x:c>
-      <x:c r="D16" s="18" t="str">
+      <x:c r="D16" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13859,7 +13868,7 @@
       <x:c r="C17" s="9" t="str">
         <x:v>1036 fish; 21.5–64.4 cm; not focal-source membership.</x:v>
       </x:c>
-      <x:c r="D17" s="18" t="str">
+      <x:c r="D17" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13873,7 +13882,7 @@
       <x:c r="C18" s="9" t="str">
         <x:v>FishBase Siganus canaliculatus/FAO Woodland; retrieved 30 September 2026.</x:v>
       </x:c>
-      <x:c r="D18" s="18" t="str">
+      <x:c r="D18" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13887,7 +13896,7 @@
       <x:c r="C19" s="9" t="str">
         <x:v>Frontiers in Marine Science(2017)4: 285; retrieved 30 September 2026.</x:v>
       </x:c>
-      <x:c r="D19" s="18" t="str">
+      <x:c r="D19" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13901,7 +13910,7 @@
       <x:c r="C20" s="9" t="str">
         <x:v>FishBase Labridae family account; retrieved 30 September 2026.</x:v>
       </x:c>
-      <x:c r="D20" s="18" t="str">
+      <x:c r="D20" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13915,7 +13924,7 @@
       <x:c r="C21" s="9" t="str">
         <x:v>FAO high-seas resource assessment, section 5.3; retrieved 30 September 2026.</x:v>
       </x:c>
-      <x:c r="D21" s="18" t="str">
+      <x:c r="D21" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13929,7 +13938,7 @@
       <x:c r="C22" s="9" t="str">
         <x:v>FishBase Lepidocybium flavobrunneum, retrieved 30 September 2026.</x:v>
       </x:c>
-      <x:c r="D22" s="18" t="str">
+      <x:c r="D22" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13943,7 +13952,7 @@
       <x:c r="C23" s="9" t="str">
         <x:v>NOAA Fisheries Opah Science; biology and research sections read 30 September 2026. CSIRO page could not be retrieved reliably.</x:v>
       </x:c>
-      <x:c r="D23" s="18" t="str">
+      <x:c r="D23" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13957,7 +13966,7 @@
       <x:c r="C24" s="9" t="str">
         <x:v>93 basic cells; 24 catch totals; 528 diet cells.</x:v>
       </x:c>
-      <x:c r="D24" s="18" t="str">
+      <x:c r="D24" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13971,7 +13980,7 @@
       <x:c r="C25" s="9" t="str">
         <x:v>See adopted_GE.json, adopted_TE.json, adopted_With_Egestion.json and adopted_provenance.json.</x:v>
       </x:c>
-      <x:c r="D25" s="18" t="str">
+      <x:c r="D25" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>
@@ -13985,7 +13994,7 @@
       <x:c r="C26" s="9" t="str">
         <x:v>Correct source figure printed p. 8/PDF 18; original LME boundary.</x:v>
       </x:c>
-      <x:c r="D26" s="18" t="str">
+      <x:c r="D26" s="19" t="str">
         <x:v>Open source</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Complete validation reviews for all 23 selected regions
Reassess taxonomy, complete candidate membership, allocation evidence and confidence while preserving accepted scientific parameters and researcher fields. Retain regional DOCX reports, linked Excel appendices and reproducible source, diagnostic and arithmetic evidence.

Reconcile selected models and annual results with Project.xlsx, map, trends and archive; make current availability distinct from diagnostic grade and scientific approval. Verify portable Office links, relocated generated pages, calculation controls and exports.

Integrate reviewed workflow lessons and refresh the knowledge graph with preserved evidence, full-byte freshness checks and all-region retrieval. Validation: 56 workflow tests, 16 verifier regression checks, all 23 protected-input/serialization and shared-output reconciliations.
</commit_message>
<xml_diff>
--- a/regions/LME_032/LME032_taxon_mapping_appendix.xlsx
+++ b/regions/LME_032/LME032_taxon_mapping_appendix.xlsx
@@ -1638,10 +1638,10 @@
         <x:v>Large Benthopelagics (99.9900%); Benthic Omnivores (0.0100%)</x:v>
       </x:c>
       <x:c r="F56" s="9" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="G56" s="9" t="str">
-        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Retained weights use identified, singly assigned total catch within this lineage in Arabian Sea 1950–2019. Its observed mix is assumed for the coarse label and held fixed across years/bases. See Sources and Allocation evidence.</x:v>
+        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Identified Arabian Sea lineage catches retain the numerical proxy split. Coarse catch is 99.99% India, while identified donors are almost entirely elsewhere; their country and gear composition differ. The residual composition is unobserved, so allocation is Low and fixed across years/bases. See Sources and Allocation evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="80" customHeight="1">
@@ -6054,10 +6054,10 @@
         <x:v>Med Benthic Carnivores (17.3452%); Benthic Omnivores (82.6548%)</x:v>
       </x:c>
       <x:c r="F248" s="9" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="G248" s="9" t="str">
-        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Retained weights use identified, singly assigned total catch within this lineage in Arabian Sea 1950–2019. Its observed mix is assumed for the coarse label and held fixed across years/bases. See Sources and Allocation evidence.</x:v>
+        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Identified Arabian Sea lineage catches retain the numerical proxy split. Coarse catch is concentrated in 1950–1979 and small-scale gillnets; identified donors mainly come from 1990–2019 and other gears. The residual composition is unobserved, so allocation is Low and fixed across years/bases. See Sources and Allocation evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="249" ht="64" customHeight="1">
@@ -10467,19 +10467,19 @@
       </x:c>
       <x:c r="B7" s="2" t="n">
         <x:f>COUNTIF('Taxon appendix'!$F$6:$F$435,A7)</x:f>
-        <x:v>207</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="C7" s="8" t="n">
         <x:f>SUMIF('Taxon appendix'!$F$6:$F$435,A7,'Taxon appendix'!$C$6:$C$435)</x:f>
-        <x:v>2580243.723961291</x:v>
+        <x:v>2534929.25610556</x:v>
       </x:c>
       <x:c r="D7" s="12" t="n">
         <x:f>100*C7/SUM('Taxon appendix'!$C$6:$C$435)</x:f>
-        <x:v>49.39498135125588</x:v>
+        <x:v>48.52750233216555</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
         <x:f>100*SUMIF('Taxon appendix'!$F$6:$F$435,A7,'Taxon appendix'!$D$6:$D$435)/SUM('Taxon appendix'!$D$6:$D$435)</x:f>
-        <x:v>64.52104397268963</x:v>
+        <x:v>64.2252681737161</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -10488,19 +10488,19 @@
       </x:c>
       <x:c r="B8" s="2" t="n">
         <x:f>COUNTIF('Taxon appendix'!$F$6:$F$435,A8)</x:f>
-        <x:v>38</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C8" s="8" t="n">
         <x:f>SUMIF('Taxon appendix'!$F$6:$F$435,A8,'Taxon appendix'!$C$6:$C$435)</x:f>
-        <x:v>167328.87029954733</x:v>
+        <x:v>212643.33815527774</x:v>
       </x:c>
       <x:c r="D8" s="12" t="n">
         <x:f>100*C8/SUM('Taxon appendix'!$C$6:$C$435)</x:f>
-        <x:v>3.203265781142483</x:v>
+        <x:v>4.0707448002328</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
         <x:f>100*SUMIF('Taxon appendix'!$F$6:$F$435,A8,'Taxon appendix'!$D$6:$D$435)/SUM('Taxon appendix'!$D$6:$D$435)</x:f>
-        <x:v>4.273403098680445</x:v>
+        <x:v>4.569178897653987</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10790,7 +10790,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="C32" s="14" t="n">
-        <x:v>6.424645933528023</x:v>
+        <x:v>6.128870134554482</x:v>
       </x:c>
       <x:c r="D32" s="2"/>
       <x:c r="E32" s="2"/>
@@ -10808,10 +10808,16 @@
       <x:c r="D33" s="2"/>
       <x:c r="E33" s="2"/>
     </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="2"/>
-      <x:c r="B34" s="2"/>
-      <x:c r="C34" s="2"/>
+    <x:row r="34" ht="38" customHeight="1">
+      <x:c r="A34" s="9" t="str">
+        <x:v>Identified regional catch composition assumed for the coarse taxon</x:v>
+      </x:c>
+      <x:c r="B34" s="9" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="C34" s="14" t="n">
+        <x:v>0.29577579897353967</x:v>
+      </x:c>
       <x:c r="D34" s="2"/>
       <x:c r="E34" s="2"/>
     </x:row>
@@ -11744,10 +11750,10 @@
         <x:v>0.9998996577124797</x:v>
       </x:c>
       <x:c r="I27" s="9" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="J27" s="9" t="str">
-        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Retained weights use identified, singly assigned total catch within this lineage in Arabian Sea 1950–2019. Its observed mix is assumed for the coarse label and held fixed across years/bases.</x:v>
+        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Identified Arabian Sea lineage catches retain the numerical proxy split. Coarse catch is 99.99% India, while identified donors are almost entirely elsewhere; their country and gear composition differ. The residual composition is unobserved, so allocation is Low and fixed across years/bases.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="80" customHeight="1">
@@ -11777,10 +11783,10 @@
         <x:v>0.00010034228752020908</x:v>
       </x:c>
       <x:c r="I28" s="9" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="J28" s="9" t="str">
-        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Retained weights use identified, singly assigned total catch within this lineage in Arabian Sea 1950–2019. Its observed mix is assumed for the coarse label and held fixed across years/bases.</x:v>
+        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Identified Arabian Sea lineage catches retain the numerical proxy split. Coarse catch is 99.99% India, while identified donors are almost entirely elsewhere; their country and gear composition differ. The residual composition is unobserved, so allocation is Low and fixed across years/bases.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="80" customHeight="1">
@@ -12635,10 +12641,10 @@
         <x:v>0.1734515964828827</x:v>
       </x:c>
       <x:c r="I54" s="9" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="J54" s="9" t="str">
-        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Retained weights use identified, singly assigned total catch within this lineage in Arabian Sea 1950–2019. Its observed mix is assumed for the coarse label and held fixed across years/bases.</x:v>
+        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Identified Arabian Sea lineage catches retain the numerical proxy split. Coarse catch is concentrated in 1950–1979 and small-scale gillnets; identified donors mainly come from 1990–2019 and other gears. The residual composition is unobserved, so allocation is Low and fixed across years/bases.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="80" customHeight="1">
@@ -12668,10 +12674,10 @@
         <x:v>0.8265484035171173</x:v>
       </x:c>
       <x:c r="I55" s="9" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Low</x:v>
       </x:c>
       <x:c r="J55" s="9" t="str">
-        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Retained weights use identified, singly assigned total catch within this lineage in Arabian Sea 1950–2019. Its observed mix is assumed for the coarse label and held fixed across years/bases.</x:v>
+        <x:v>The named lineage spans the source compartments; use identified regional members as a composition proxy, rather than assign the whole label to one guild. Identified Arabian Sea lineage catches retain the numerical proxy split. Coarse catch is concentrated in 1950–1979 and small-scale gillnets; identified donors mainly come from 1990–2019 and other gears. The residual composition is unobserved, so allocation is Low and fixed across years/bases.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="64" customHeight="1">
@@ -13996,6 +14002,20 @@
       </x:c>
       <x:c r="D26" s="19" t="str">
         <x:v>Open source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="56" customHeight="1">
+      <x:c r="A27" t="str" s="9">
+        <x:v>Reporting applicability review</x:v>
+      </x:c>
+      <x:c r="B27" t="str" s="9">
+        <x:v>SAU v50.1 donor/target country, sector, gear and period comparison; 30 September 2026</x:v>
+      </x:c>
+      <x:c r="C27" t="str" s="9">
+        <x:v>Siluriformes and Pleuronectiformes retain numerical weights at Low allocation confidence</x:v>
+      </x:c>
+      <x:c r="D27" t="str" s="19">
+        <x:v>Open evidence</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14026,6 +14046,7 @@
     <x:hyperlink xmlns:ns20="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" ns20:id="rIdHyperlink20"/>
     <x:hyperlink xmlns:ns21="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" ns21:id="rIdHyperlink21"/>
     <x:hyperlink xmlns:ns22="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" ns22:id="rIdHyperlink22"/>
+    <x:hyperlink xmlns:ns0="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" ns0:id="rIdReportingApplicability"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">

</xml_diff>